<commit_message>
updated on sep 12
</commit_message>
<xml_diff>
--- a/12628474.xlsx
+++ b/12628474.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="70">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2259,26 +2259,48 @@
       </c>
     </row>
     <row r="19" spans="1:14">
-      <c r="A19" s="18"/>
+      <c r="A19" s="18">
+        <v>46277</v>
+      </c>
       <c r="B19" s="19"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="19"/>
-      <c r="H19" s="19"/>
-      <c r="I19" s="15" t="str">
+      <c r="C19" s="19">
+        <v>20</v>
+      </c>
+      <c r="D19" s="19">
+        <v>120</v>
+      </c>
+      <c r="E19" s="19">
+        <v>30</v>
+      </c>
+      <c r="F19" s="19">
+        <v>0</v>
+      </c>
+      <c r="G19" s="19">
+        <v>0</v>
+      </c>
+      <c r="H19" s="19">
+        <v>400</v>
+      </c>
+      <c r="I19" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J19" s="15" t="str">
+        <v>570</v>
+      </c>
+      <c r="J19" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K19" s="20"/>
-      <c r="L19" s="20"/>
-      <c r="M19" s="20"/>
-      <c r="N19" s="21"/>
+        <v>870</v>
+      </c>
+      <c r="K19" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="L19" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="M19" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="N19" s="21" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="18"/>

</xml_diff>